<commit_message>
rebuilt tables and fixed discaRd issues
-rebuilt obs_prorate table
-rebuilt cams_catch_mock
-added region/halfofyear to mimic ACL accounting
-ran tests to compare squids against ACL accounting 2019
-identified issues with previous code using incorrect column for trip counts..
-KALL is relatively unaffected
-overall, illex is fairly close. seeing a drop in discard estimate but an increase in CV
-developed end to end run scheme making most things into functions

Co-Authored-By: Dan <danlinden@gmail.com>
</commit_message>
<xml_diff>
--- a/CAMS/SMB_FY2019_discRd_BG_example.xlsx
+++ b/CAMS/SMB_FY2019_discRd_BG_example.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="mack" sheetId="1" r:id="rId1"/>
@@ -323,12 +323,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -343,11 +349,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1396,25 +1403,25 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="A30" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="2">
         <v>1750</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="2">
         <v>122</v>
       </c>
-      <c r="D30">
+      <c r="D30" s="2">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="2">
         <v>1.458214441496547E-2</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="2">
         <v>21896431.973870799</v>
       </c>
-      <c r="G30">
+      <c r="G30" s="2">
         <v>319296.93321545131</v>
       </c>
       <c r="H30">
@@ -1434,25 +1441,25 @@
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="A31" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="2">
         <v>3019</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="2">
         <v>375</v>
       </c>
-      <c r="D31">
+      <c r="D31" s="2">
         <v>0.12</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="2">
         <v>4.0658350804005754E-3</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="2">
         <v>25577560.136865132</v>
       </c>
-      <c r="G31">
+      <c r="G31" s="2">
         <v>103994.1412755216</v>
       </c>
       <c r="H31">
@@ -1460,25 +1467,25 @@
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="A32" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="2">
         <v>2530</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="2">
         <v>211</v>
       </c>
-      <c r="D32">
+      <c r="D32" s="2">
         <v>0.08</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="2">
         <v>1.6048277985198369E-3</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="2">
         <v>29024889.379979141</v>
       </c>
-      <c r="G32">
+      <c r="G32" s="2">
         <v>46579.949325953712</v>
       </c>
       <c r="H32">
@@ -1486,25 +1493,25 @@
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="A33" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="2">
         <v>2346</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="2">
         <v>432</v>
       </c>
-      <c r="D33">
+      <c r="D33" s="2">
         <v>0.18</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="2">
         <v>9.3894767853846484E-5</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="2">
         <v>33392176.301814649</v>
       </c>
-      <c r="G33">
+      <c r="G33" s="2">
         <v>3135.3506419936002</v>
       </c>
       <c r="H33">
@@ -4447,6 +4454,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="40.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -5173,106 +5184,106 @@
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="A30" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="2">
         <v>1750</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="2">
         <v>122</v>
       </c>
-      <c r="D30">
+      <c r="D30" s="2">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="2">
         <v>2.1118282427345699E-3</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="2">
         <v>21896431.973870799</v>
       </c>
-      <c r="G30">
+      <c r="G30" s="2">
         <v>46241.503457536608</v>
       </c>
-      <c r="H30">
+      <c r="H30" s="2">
         <v>0.41</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="A31" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="2">
         <v>3019</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="2">
         <v>375</v>
       </c>
-      <c r="D31">
+      <c r="D31" s="2">
         <v>0.12</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="2">
         <v>2.000886788871856E-2</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="2">
         <v>25577560.136865132</v>
       </c>
-      <c r="G31">
+      <c r="G31" s="2">
         <v>511778.02169428871</v>
       </c>
-      <c r="H31">
+      <c r="H31" s="2">
         <v>0.34</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="A32" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="2">
         <v>2530</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="2">
         <v>211</v>
       </c>
-      <c r="D32">
+      <c r="D32" s="2">
         <v>0.08</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="2">
         <v>5.5523334435985628E-3</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="2">
         <v>29024889.379979141</v>
       </c>
-      <c r="G32">
+      <c r="G32" s="2">
         <v>161155.86400120691</v>
       </c>
-      <c r="H32">
+      <c r="H32" s="2">
         <v>0.48</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="A33" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="2">
         <v>2346</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="2">
         <v>432</v>
       </c>
-      <c r="D33">
+      <c r="D33" s="2">
         <v>0.18</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="2">
         <v>2.5940985172919042E-3</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="2">
         <v>33392176.301814649</v>
       </c>
-      <c r="G33">
+      <c r="G33" s="2">
         <v>86622.595033687234</v>
       </c>
-      <c r="H33">
+      <c r="H33" s="2">
         <v>0.31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
exploring mesh mismatches between obs and VTR
see the bottom of the MSB V2 module... it's significant
</commit_message>
<xml_diff>
--- a/CAMS/SMB_FY2019_discRd_BG_example.xlsx
+++ b/CAMS/SMB_FY2019_discRd_BG_example.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="2"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="mack" sheetId="1" r:id="rId1"/>
@@ -306,7 +306,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -316,6 +320,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,17 +357,24 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -663,6 +681,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -682,10 +702,10 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -708,10 +728,10 @@
       <c r="E2">
         <v>0</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="3">
         <v>2300</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="3">
         <v>0</v>
       </c>
     </row>
@@ -731,10 +751,10 @@
       <c r="E3">
         <v>0</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="3">
         <v>21469.262905162061</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="3">
         <v>0</v>
       </c>
     </row>
@@ -754,10 +774,10 @@
       <c r="E4">
         <v>0</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="3">
         <v>753569.72512978013</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="3">
         <v>0</v>
       </c>
       <c r="H4">
@@ -780,10 +800,10 @@
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="3">
         <v>700962.931795649</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="3">
         <v>0</v>
       </c>
       <c r="H5">
@@ -806,10 +826,10 @@
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="3">
         <v>2452355.66145615</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="3">
         <v>0</v>
       </c>
       <c r="H6">
@@ -832,10 +852,10 @@
       <c r="E7">
         <v>0</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="3">
         <v>1761815.053452285</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="3">
         <v>0</v>
       </c>
       <c r="H7">
@@ -858,10 +878,10 @@
       <c r="E8">
         <v>0</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="3">
         <v>824600.54603952006</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="3">
         <v>0</v>
       </c>
       <c r="H8">
@@ -884,10 +904,10 @@
       <c r="E9">
         <v>0</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="3">
         <v>342935.35396048002</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="3">
         <v>0</v>
       </c>
       <c r="H9">
@@ -910,10 +930,10 @@
       <c r="E10">
         <v>0</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="3">
         <v>3597855.4026433248</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="3">
         <v>0</v>
       </c>
       <c r="H10">
@@ -936,10 +956,10 @@
       <c r="E11">
         <v>0</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="3">
         <v>371539.38865177229</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="3">
         <v>0</v>
       </c>
       <c r="H11">
@@ -962,10 +982,10 @@
       <c r="E12">
         <v>2.6749104259039591E-6</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="3">
         <v>2478138.821705427</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="3">
         <v>6.6287993710171964</v>
       </c>
     </row>
@@ -985,10 +1005,10 @@
       <c r="E13">
         <v>1.158192941045663E-6</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="3">
         <v>18322212.479166672</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="3">
         <v>21.220657157709589</v>
       </c>
       <c r="H13">
@@ -1011,10 +1031,10 @@
       <c r="E14">
         <v>2.6749104259039591E-6</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="3">
         <v>6774519.576923077</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="3">
         <v>18.121233046802018</v>
       </c>
       <c r="H14">
@@ -1037,10 +1057,10 @@
       <c r="E15">
         <v>1.158192941045663E-6</v>
       </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15">
+      <c r="F15" s="3">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1060,10 +1080,10 @@
       <c r="E16">
         <v>0</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="3">
         <v>38844786.131999999</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="3">
         <v>0</v>
       </c>
       <c r="H16">
@@ -1086,10 +1106,10 @@
       <c r="E17">
         <v>0</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="3">
         <v>15722</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1109,10 +1129,10 @@
       <c r="E18">
         <v>0</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="3">
         <v>23373052.6192853</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="3">
         <v>0</v>
       </c>
       <c r="H18">
@@ -1135,10 +1155,10 @@
       <c r="E19">
         <v>0</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="3">
         <v>117464020.329</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="3">
         <v>0</v>
       </c>
       <c r="H19">
@@ -1161,10 +1181,10 @@
       <c r="E20">
         <v>0</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="3">
         <v>160428</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1184,10 +1204,10 @@
       <c r="E21">
         <v>0</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="3">
         <v>22473219.009149559</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="3">
         <v>0</v>
       </c>
       <c r="H21">
@@ -1210,10 +1230,10 @@
       <c r="E22">
         <v>2.2426049611471639E-4</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="3">
         <v>36428091.839511126</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="3">
         <v>8169.3819484412188</v>
       </c>
       <c r="H22">
@@ -1248,10 +1268,10 @@
       <c r="E23">
         <v>9.0540010726617291E-5</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="3">
         <v>6906618.0694853142</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="3">
         <v>625.32527409584918</v>
       </c>
       <c r="H23">
@@ -1274,10 +1294,10 @@
       <c r="E24">
         <v>7.1636957749213769E-6</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="3">
         <v>31698095.08031968</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="3">
         <v>227.07550979994221</v>
       </c>
       <c r="H24">
@@ -1300,10 +1320,10 @@
       <c r="E25">
         <v>6.8115412806709478E-5</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="3">
         <v>6413896.8770221323</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="3">
         <v>436.88523347802732</v>
       </c>
       <c r="H25">
@@ -1326,10 +1346,10 @@
       <c r="E26">
         <v>7.4032024555400911E-3</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="3">
         <v>246476.5</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="3">
         <v>1824.7154300329271</v>
       </c>
     </row>
@@ -1349,10 +1369,10 @@
       <c r="E27">
         <v>2.0781875455635969E-3</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="3">
         <v>107667</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="3">
         <v>223.75221846819571</v>
       </c>
     </row>
@@ -1372,10 +1392,10 @@
       <c r="E28">
         <v>1.6048277985198369E-3</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="3">
         <v>68683.310872100425</v>
       </c>
-      <c r="G28">
+      <c r="G28" s="3">
         <v>110.2248865819265</v>
       </c>
     </row>
@@ -1395,10 +1415,10 @@
       <c r="E29">
         <v>6.8115412806709478E-5</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="3">
         <v>159857</v>
       </c>
-      <c r="G29">
+      <c r="G29" s="3">
         <v>10.88872554504216</v>
       </c>
     </row>
@@ -1418,10 +1438,10 @@
       <c r="E30" s="2">
         <v>1.458214441496547E-2</v>
       </c>
-      <c r="F30" s="2">
+      <c r="F30" s="5">
         <v>21896431.973870799</v>
       </c>
-      <c r="G30" s="2">
+      <c r="G30" s="5">
         <v>319296.93321545131</v>
       </c>
       <c r="H30">
@@ -1456,10 +1476,10 @@
       <c r="E31" s="2">
         <v>4.0658350804005754E-3</v>
       </c>
-      <c r="F31" s="2">
+      <c r="F31" s="5">
         <v>25577560.136865132</v>
       </c>
-      <c r="G31" s="2">
+      <c r="G31" s="5">
         <v>103994.1412755216</v>
       </c>
       <c r="H31">
@@ -1482,10 +1502,10 @@
       <c r="E32" s="2">
         <v>1.6048277985198369E-3</v>
       </c>
-      <c r="F32" s="2">
+      <c r="F32" s="5">
         <v>29024889.379979141</v>
       </c>
-      <c r="G32" s="2">
+      <c r="G32" s="5">
         <v>46579.949325953712</v>
       </c>
       <c r="H32">
@@ -1508,10 +1528,10 @@
       <c r="E33" s="2">
         <v>9.3894767853846484E-5</v>
       </c>
-      <c r="F33" s="2">
+      <c r="F33" s="5">
         <v>33392176.301814649</v>
       </c>
-      <c r="G33" s="2">
+      <c r="G33" s="5">
         <v>3135.3506419936002</v>
       </c>
       <c r="H33">
@@ -1534,10 +1554,10 @@
       <c r="E34">
         <v>8.7544303628549482E-5</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="3">
         <v>2017068.655317503</v>
       </c>
-      <c r="G34">
+      <c r="G34" s="3">
         <v>176.5828708007455</v>
       </c>
       <c r="H34">
@@ -1560,10 +1580,10 @@
       <c r="E35">
         <v>0</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="3">
         <v>2115740.8440453699</v>
       </c>
-      <c r="G35">
+      <c r="G35" s="3">
         <v>0</v>
       </c>
       <c r="H35">
@@ -1590,10 +1610,10 @@
       <c r="E36">
         <v>0</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="3">
         <v>564901.33666130423</v>
       </c>
-      <c r="G36">
+      <c r="G36" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1613,10 +1633,10 @@
       <c r="E37">
         <v>0</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="3">
         <v>152326.6300376268</v>
       </c>
-      <c r="G37">
+      <c r="G37" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1636,10 +1656,10 @@
       <c r="E38">
         <v>0</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="3">
         <v>1264097.995133939</v>
       </c>
-      <c r="G38">
+      <c r="G38" s="3">
         <v>0</v>
       </c>
       <c r="H38">
@@ -1662,10 +1682,10 @@
       <c r="E39">
         <v>0</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="3">
         <v>167204.17654073989</v>
       </c>
-      <c r="G39">
+      <c r="G39" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1685,10 +1705,10 @@
       <c r="E40">
         <v>3.3897660134232321E-4</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="3">
         <v>1519335.2860000001</v>
       </c>
-      <c r="G40">
+      <c r="G40" s="3">
         <v>515.01911154774666</v>
       </c>
       <c r="H40">
@@ -1711,10 +1731,10 @@
       <c r="E41">
         <v>2.69092083310909E-5</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="3">
         <v>19051</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="3">
         <v>0.51264732791561285</v>
       </c>
     </row>
@@ -1734,10 +1754,10 @@
       <c r="E42">
         <v>2.69092083310909E-5</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="3">
         <v>564641.01</v>
       </c>
-      <c r="G42">
+      <c r="G42" s="3">
         <v>15.19404257036758</v>
       </c>
       <c r="H42">
@@ -1760,10 +1780,10 @@
       <c r="E43">
         <v>0</v>
       </c>
-      <c r="F43">
+      <c r="F43" s="3">
         <v>31608</v>
       </c>
-      <c r="G43">
+      <c r="G43" s="3">
         <v>0</v>
       </c>
       <c r="H43">
@@ -1786,10 +1806,10 @@
       <c r="E44">
         <v>0</v>
       </c>
-      <c r="F44">
+      <c r="F44" s="3">
         <v>202455.1253333333</v>
       </c>
-      <c r="G44">
+      <c r="G44" s="3">
         <v>0</v>
       </c>
       <c r="H44">
@@ -1812,10 +1832,10 @@
       <c r="E45">
         <v>0</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="3">
         <v>301461.19276470592</v>
       </c>
-      <c r="G45">
+      <c r="G45" s="3">
         <v>0</v>
       </c>
       <c r="H45">
@@ -1838,10 +1858,10 @@
       <c r="E46">
         <v>0</v>
       </c>
-      <c r="F46">
+      <c r="F46" s="3">
         <v>248842.38373118901</v>
       </c>
-      <c r="G46">
+      <c r="G46" s="3">
         <v>0</v>
       </c>
       <c r="H46">
@@ -1864,10 +1884,10 @@
       <c r="E47">
         <v>0</v>
       </c>
-      <c r="F47">
+      <c r="F47" s="3">
         <v>792319</v>
       </c>
-      <c r="G47">
+      <c r="G47" s="3">
         <v>0</v>
       </c>
       <c r="H47">
@@ -1890,10 +1910,10 @@
       <c r="E48">
         <v>0</v>
       </c>
-      <c r="F48">
+      <c r="F48" s="3">
         <v>1172545</v>
       </c>
-      <c r="G48">
+      <c r="G48" s="3">
         <v>0</v>
       </c>
       <c r="H48">
@@ -1916,10 +1936,10 @@
       <c r="E49">
         <v>0</v>
       </c>
-      <c r="F49">
+      <c r="F49" s="3">
         <v>1892795</v>
       </c>
-      <c r="G49">
+      <c r="G49" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1939,10 +1959,10 @@
       <c r="E50">
         <v>0</v>
       </c>
-      <c r="F50">
+      <c r="F50" s="3">
         <v>20798650</v>
       </c>
-      <c r="G50">
+      <c r="G50" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1962,10 +1982,10 @@
       <c r="E51">
         <v>0</v>
       </c>
-      <c r="F51">
+      <c r="F51" s="3">
         <v>12748261</v>
       </c>
-      <c r="G51">
+      <c r="G51" s="3">
         <v>0</v>
       </c>
       <c r="H51">
@@ -1988,10 +2008,10 @@
       <c r="E52">
         <v>0</v>
       </c>
-      <c r="F52">
+      <c r="F52" s="3">
         <v>11330218</v>
       </c>
-      <c r="G52">
+      <c r="G52" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2011,10 +2031,10 @@
       <c r="E53">
         <v>2.9647301005011441E-7</v>
       </c>
-      <c r="F53">
+      <c r="F53" s="3">
         <v>184727530.00525001</v>
       </c>
-      <c r="G53">
+      <c r="G53" s="3">
         <v>54.766726859779283</v>
       </c>
       <c r="H53">
@@ -2037,10 +2057,10 @@
       <c r="E54">
         <v>5.8254710335500052E-7</v>
       </c>
-      <c r="F54">
+      <c r="F54" s="3">
         <v>79784042.78475</v>
       </c>
-      <c r="G54">
+      <c r="G54" s="3">
         <v>46.477963018207539</v>
       </c>
       <c r="H54">
@@ -2063,10 +2083,10 @@
       <c r="E55">
         <v>0</v>
       </c>
-      <c r="F55">
+      <c r="F55" s="3">
         <v>132614577.92729621</v>
       </c>
-      <c r="G55">
+      <c r="G55" s="3">
         <v>0</v>
       </c>
       <c r="H55">
@@ -2089,10 +2109,10 @@
       <c r="E56">
         <v>0</v>
       </c>
-      <c r="F56">
+      <c r="F56" s="3">
         <v>105493361.5907038</v>
       </c>
-      <c r="G56">
+      <c r="G56" s="3">
         <v>0</v>
       </c>
       <c r="H56">
@@ -2115,10 +2135,10 @@
       <c r="E57">
         <v>2.4976470083808548E-5</v>
       </c>
-      <c r="F57">
+      <c r="F57" s="3">
         <v>156123</v>
       </c>
-      <c r="G57">
+      <c r="G57" s="3">
         <v>3.8994014388944409</v>
       </c>
     </row>
@@ -2138,10 +2158,10 @@
       <c r="E58">
         <v>2.4976470083808548E-5</v>
       </c>
-      <c r="F58">
+      <c r="F58" s="3">
         <v>438704.72200000001</v>
       </c>
-      <c r="G58">
+      <c r="G58" s="3">
         <v>10.957295364658551</v>
       </c>
       <c r="H58">
@@ -2164,10 +2184,10 @@
       <c r="E59">
         <v>0</v>
       </c>
-      <c r="F59">
+      <c r="F59" s="3">
         <v>640539.32499999995</v>
       </c>
-      <c r="G59">
+      <c r="G59" s="3">
         <v>0</v>
       </c>
       <c r="H59">
@@ -2190,10 +2210,10 @@
       <c r="E60">
         <v>0</v>
       </c>
-      <c r="F60">
+      <c r="F60" s="3">
         <v>79528</v>
       </c>
-      <c r="G60">
+      <c r="G60" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2213,10 +2233,10 @@
       <c r="E61">
         <v>0</v>
       </c>
-      <c r="F61">
+      <c r="F61" s="3">
         <v>619909.95116279065</v>
       </c>
-      <c r="G61">
+      <c r="G61" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2236,10 +2256,10 @@
       <c r="E62">
         <v>0</v>
       </c>
-      <c r="F62">
+      <c r="F62" s="3">
         <v>62199.4</v>
       </c>
-      <c r="G62">
+      <c r="G62" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2259,10 +2279,10 @@
       <c r="E63">
         <v>0</v>
       </c>
-      <c r="F63">
+      <c r="F63" s="3">
         <v>492005.245</v>
       </c>
-      <c r="G63">
+      <c r="G63" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2282,10 +2302,10 @@
       <c r="E64">
         <v>2.707053483513985E-3</v>
       </c>
-      <c r="F64">
+      <c r="F64" s="3">
         <v>913348.23580446152</v>
       </c>
-      <c r="G64">
+      <c r="G64" s="3">
         <v>2472.48252339582</v>
       </c>
       <c r="H64">
@@ -2308,10 +2328,10 @@
       <c r="E65">
         <v>1.0600144396854239E-4</v>
       </c>
-      <c r="F65">
+      <c r="F65" s="3">
         <v>5900901.001218589</v>
       </c>
-      <c r="G65">
+      <c r="G65" s="3">
         <v>625.50402684458811</v>
       </c>
       <c r="H65">
@@ -2334,10 +2354,10 @@
       <c r="E66">
         <v>1.9758218340006759E-4</v>
       </c>
-      <c r="F66">
+      <c r="F66" s="3">
         <v>4739632.0318539664</v>
       </c>
-      <c r="G66">
+      <c r="G66" s="3">
         <v>936.46684536660541</v>
       </c>
       <c r="H66">
@@ -2360,10 +2380,10 @@
       <c r="E67">
         <v>6.9335785601398478E-6</v>
       </c>
-      <c r="F67">
+      <c r="F67" s="3">
         <v>4326410.9030381572</v>
       </c>
-      <c r="G67">
+      <c r="G67" s="3">
         <v>29.99750987966064</v>
       </c>
       <c r="H67">
@@ -2386,10 +2406,10 @@
       <c r="E68">
         <v>1.367946279792067E-3</v>
       </c>
-      <c r="F68">
+      <c r="F68" s="3">
         <v>17226.322559848741</v>
       </c>
-      <c r="G68">
+      <c r="G68" s="3">
         <v>23.56468386024325</v>
       </c>
     </row>
@@ -2409,10 +2429,10 @@
       <c r="E69">
         <v>5.4513088380210083E-5</v>
       </c>
-      <c r="F69">
+      <c r="F69" s="3">
         <v>93717.001999999993</v>
       </c>
-      <c r="G69">
+      <c r="G69" s="3">
         <v>5.1088032127543244</v>
       </c>
     </row>
@@ -2432,10 +2452,10 @@
       <c r="E70">
         <v>1.245375624931868E-4</v>
       </c>
-      <c r="F70">
+      <c r="F70" s="3">
         <v>88026.33906281479</v>
       </c>
-      <c r="G70">
+      <c r="G70" s="3">
         <v>10.96258570208175</v>
       </c>
     </row>
@@ -2455,10 +2475,10 @@
       <c r="E71">
         <v>3.4667892800699239E-6</v>
       </c>
-      <c r="F71">
+      <c r="F71" s="3">
         <v>27117.873653330069</v>
       </c>
-      <c r="G71">
+      <c r="G71" s="3">
         <v>9.40119536796553E-2</v>
       </c>
     </row>
@@ -2478,10 +2498,10 @@
       <c r="E72">
         <v>2.8839076070148979E-5</v>
       </c>
-      <c r="F72">
+      <c r="F72" s="3">
         <v>8190024.8600657582</v>
       </c>
-      <c r="G72">
+      <c r="G72" s="3">
         <v>236.19274995584769</v>
       </c>
       <c r="H72">
@@ -2504,10 +2524,10 @@
       <c r="E73">
         <v>3.0247327918777401E-6</v>
       </c>
-      <c r="F73">
+      <c r="F73" s="3">
         <v>4353366.5807391303</v>
       </c>
-      <c r="G73">
+      <c r="G73" s="3">
         <v>13.16777065182632</v>
       </c>
       <c r="H73">
@@ -2530,10 +2550,10 @@
       <c r="E74">
         <v>5.1492941586306003E-5</v>
       </c>
-      <c r="F74">
+      <c r="F74" s="3">
         <v>10837196.79415895</v>
       </c>
-      <c r="G74">
+      <c r="G74" s="3">
         <v>558.03914148092917</v>
       </c>
       <c r="H74">
@@ -2556,10 +2576,10 @@
       <c r="E75">
         <v>0</v>
       </c>
-      <c r="F75">
+      <c r="F75" s="3">
         <v>2139314.2969999998</v>
       </c>
-      <c r="G75">
+      <c r="G75" s="3">
         <v>0</v>
       </c>
       <c r="H75">
@@ -2575,6 +2595,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="15.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -2592,10 +2616,10 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -2618,10 +2642,10 @@
       <c r="E2">
         <v>0</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="3">
         <v>2300</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2641,10 +2665,10 @@
       <c r="E3">
         <v>0</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="3">
         <v>21469.262905162061</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2664,10 +2688,10 @@
       <c r="E4">
         <v>0</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="3">
         <v>753569.72512978013</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="3">
         <v>0</v>
       </c>
       <c r="H4">
@@ -2690,10 +2714,10 @@
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="3">
         <v>700962.931795649</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="3">
         <v>0</v>
       </c>
       <c r="H5">
@@ -2716,10 +2740,10 @@
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="3">
         <v>2452355.66145615</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="3">
         <v>0</v>
       </c>
       <c r="H6">
@@ -2742,10 +2766,10 @@
       <c r="E7">
         <v>0</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="3">
         <v>1761815.053452285</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="3">
         <v>0</v>
       </c>
       <c r="H7">
@@ -2768,10 +2792,10 @@
       <c r="E8">
         <v>0</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="3">
         <v>824600.54603952006</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="3">
         <v>0</v>
       </c>
       <c r="H8">
@@ -2794,10 +2818,10 @@
       <c r="E9">
         <v>0</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="3">
         <v>342935.35396048002</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="3">
         <v>0</v>
       </c>
       <c r="H9">
@@ -2820,10 +2844,10 @@
       <c r="E10">
         <v>0</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="3">
         <v>3597855.4026433248</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="3">
         <v>0</v>
       </c>
       <c r="H10">
@@ -2846,10 +2870,10 @@
       <c r="E11">
         <v>0</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="3">
         <v>371539.38865177229</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="3">
         <v>0</v>
       </c>
       <c r="H11">
@@ -2872,10 +2896,10 @@
       <c r="E12">
         <v>3.9336918027999386E-6</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="3">
         <v>2478138.821705427</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="3">
         <v>9.7482343691429367</v>
       </c>
     </row>
@@ -2895,10 +2919,10 @@
       <c r="E13">
         <v>0</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="3">
         <v>18322212.479166672</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="3">
         <v>0</v>
       </c>
       <c r="H13">
@@ -2921,10 +2945,10 @@
       <c r="E14">
         <v>3.9336918027999386E-6</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="3">
         <v>6774519.576923077</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="3">
         <v>26.648872127650019</v>
       </c>
       <c r="H14">
@@ -2947,10 +2971,10 @@
       <c r="E15">
         <v>0</v>
       </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15">
+      <c r="F15" s="3">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2970,10 +2994,10 @@
       <c r="E16">
         <v>0</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="3">
         <v>38844786.131999999</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="3">
         <v>0</v>
       </c>
       <c r="H16">
@@ -2996,10 +3020,10 @@
       <c r="E17">
         <v>0</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="3">
         <v>15722</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3019,10 +3043,10 @@
       <c r="E18">
         <v>0</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="3">
         <v>23373052.6192853</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="3">
         <v>0</v>
       </c>
       <c r="H18">
@@ -3045,10 +3069,10 @@
       <c r="E19">
         <v>0</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="3">
         <v>117464020.329</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="3">
         <v>0</v>
       </c>
       <c r="H19">
@@ -3071,10 +3095,10 @@
       <c r="E20">
         <v>0</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="3">
         <v>160428</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3094,10 +3118,10 @@
       <c r="E21">
         <v>0</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="3">
         <v>22473219.009149559</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="3">
         <v>0</v>
       </c>
       <c r="H21">
@@ -3120,10 +3144,10 @@
       <c r="E22">
         <v>1.3946194039676191E-4</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="3">
         <v>36428091.839511126</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="3">
         <v>5080.3323728896694</v>
       </c>
       <c r="H22">
@@ -3146,10 +3170,10 @@
       <c r="E23">
         <v>1.0415637952730001E-4</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="3">
         <v>6906618.0694853142</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="3">
         <v>719.36833289542005</v>
       </c>
       <c r="H23">
@@ -3172,10 +3196,10 @@
       <c r="E24">
         <v>1.5174450171877381E-3</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="3">
         <v>31698095.08031968</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="3">
         <v>48100.116433974232</v>
       </c>
       <c r="H24">
@@ -3198,10 +3222,10 @@
       <c r="E25">
         <v>9.567656249728559E-5</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="3">
         <v>6413896.8770221323</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="3">
         <v>613.65960540555295</v>
       </c>
       <c r="H25">
@@ -3224,10 +3248,10 @@
       <c r="E26">
         <v>5.1474061031380122E-3</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="3">
         <v>246476.5</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="3">
         <v>1268.7146403800959</v>
       </c>
     </row>
@@ -3247,10 +3271,10 @@
       <c r="E27">
         <v>3.2182618238282307E-2</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="3">
         <v>107667</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="3">
         <v>3465.0059578611422</v>
       </c>
     </row>
@@ -3270,10 +3294,10 @@
       <c r="E28">
         <v>5.3620337599451307E-3</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="3">
         <v>68683.310872100425</v>
       </c>
-      <c r="G28">
+      <c r="G28" s="3">
         <v>368.28223164100888</v>
       </c>
     </row>
@@ -3293,10 +3317,10 @@
       <c r="E29">
         <v>9.567656249728559E-5</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="3">
         <v>159857</v>
       </c>
-      <c r="G29">
+      <c r="G29" s="3">
         <v>15.294568251128579</v>
       </c>
     </row>
@@ -3316,10 +3340,10 @@
       <c r="E30">
         <v>1.015535026587926E-2</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="3">
         <v>21896431.973870799</v>
       </c>
-      <c r="G30">
+      <c r="G30" s="3">
         <v>222365.93626765601</v>
       </c>
       <c r="H30">
@@ -3342,10 +3366,10 @@
       <c r="E31">
         <v>6.4261080097037321E-2</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="3">
         <v>25577560.136865132</v>
       </c>
-      <c r="G31">
+      <c r="G31" s="3">
         <v>1643641.6406418791</v>
       </c>
       <c r="H31">
@@ -3368,10 +3392,10 @@
       <c r="E32">
         <v>5.3620337599451307E-3</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="3">
         <v>29024889.379979141</v>
       </c>
-      <c r="G32">
+      <c r="G32" s="3">
         <v>155632.43673412109</v>
       </c>
       <c r="H32">
@@ -3394,10 +3418,10 @@
       <c r="E33">
         <v>5.4160942132072979E-3</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="3">
         <v>33392176.301814649</v>
       </c>
-      <c r="G33">
+      <c r="G33" s="3">
         <v>180855.1728346562</v>
       </c>
       <c r="H33">
@@ -3420,10 +3444,10 @@
       <c r="E34">
         <v>3.8769620178357632E-4</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="3">
         <v>2017068.655317503</v>
       </c>
-      <c r="G34">
+      <c r="G34" s="3">
         <v>782.00985640330168</v>
       </c>
       <c r="H34">
@@ -3446,10 +3470,10 @@
       <c r="E35">
         <v>1.39005339277192E-2</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="3">
         <v>2115740.8440453699</v>
       </c>
-      <c r="G35">
+      <c r="G35" s="3">
         <v>29409.927384913921</v>
       </c>
       <c r="H35">
@@ -3472,10 +3496,10 @@
       <c r="E36">
         <v>6.4650379368426131E-2</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="3">
         <v>564901.33666130423</v>
       </c>
-      <c r="G36">
+      <c r="G36" s="3">
         <v>36521.08572088433</v>
       </c>
     </row>
@@ -3495,10 +3519,10 @@
       <c r="E37">
         <v>6.4650379368426131E-2</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="3">
         <v>152326.6300376268</v>
       </c>
-      <c r="G37">
+      <c r="G37" s="3">
         <v>9847.9744198464668</v>
       </c>
     </row>
@@ -3518,10 +3542,10 @@
       <c r="E38">
         <v>6.4650379368426131E-2</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="3">
         <v>1264097.995133939</v>
       </c>
-      <c r="G38">
+      <c r="G38" s="3">
         <v>81724.414944276039</v>
       </c>
     </row>
@@ -3541,10 +3565,10 @@
       <c r="E39">
         <v>6.4650379368426131E-2</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="3">
         <v>167204.17654073989</v>
       </c>
-      <c r="G39">
+      <c r="G39" s="3">
         <v>10809.813445344131</v>
       </c>
     </row>
@@ -3564,10 +3588,10 @@
       <c r="E40">
         <v>0.1799706854480175</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="3">
         <v>1519335.2860000001</v>
       </c>
-      <c r="G40">
+      <c r="G40" s="3">
         <v>273435.81284677971</v>
       </c>
       <c r="H40">
@@ -3590,10 +3614,10 @@
       <c r="E41">
         <v>0</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="3">
         <v>19051</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3613,10 +3637,10 @@
       <c r="E42">
         <v>0</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="3">
         <v>564641.01</v>
       </c>
-      <c r="G42">
+      <c r="G42" s="3">
         <v>0</v>
       </c>
       <c r="H42">
@@ -3639,10 +3663,10 @@
       <c r="E43">
         <v>0</v>
       </c>
-      <c r="F43">
+      <c r="F43" s="3">
         <v>31608</v>
       </c>
-      <c r="G43">
+      <c r="G43" s="3">
         <v>0</v>
       </c>
       <c r="H43">
@@ -3665,10 +3689,10 @@
       <c r="E44">
         <v>0</v>
       </c>
-      <c r="F44">
+      <c r="F44" s="3">
         <v>202455.1253333333</v>
       </c>
-      <c r="G44">
+      <c r="G44" s="3">
         <v>0</v>
       </c>
       <c r="H44">
@@ -3691,10 +3715,10 @@
       <c r="E45">
         <v>0</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="3">
         <v>301461.19276470592</v>
       </c>
-      <c r="G45">
+      <c r="G45" s="3">
         <v>0</v>
       </c>
       <c r="H45">
@@ -3717,10 +3741,10 @@
       <c r="E46">
         <v>0</v>
       </c>
-      <c r="F46">
+      <c r="F46" s="3">
         <v>248842.38373118901</v>
       </c>
-      <c r="G46">
+      <c r="G46" s="3">
         <v>0</v>
       </c>
       <c r="H46">
@@ -3743,10 +3767,10 @@
       <c r="E47">
         <v>0</v>
       </c>
-      <c r="F47">
+      <c r="F47" s="3">
         <v>792319</v>
       </c>
-      <c r="G47">
+      <c r="G47" s="3">
         <v>0</v>
       </c>
       <c r="H47">
@@ -3769,10 +3793,10 @@
       <c r="E48">
         <v>0</v>
       </c>
-      <c r="F48">
+      <c r="F48" s="3">
         <v>1172545</v>
       </c>
-      <c r="G48">
+      <c r="G48" s="3">
         <v>0</v>
       </c>
       <c r="H48">
@@ -3795,10 +3819,10 @@
       <c r="E49">
         <v>0</v>
       </c>
-      <c r="F49">
+      <c r="F49" s="3">
         <v>1892795</v>
       </c>
-      <c r="G49">
+      <c r="G49" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3818,10 +3842,10 @@
       <c r="E50">
         <v>0</v>
       </c>
-      <c r="F50">
+      <c r="F50" s="3">
         <v>20798650</v>
       </c>
-      <c r="G50">
+      <c r="G50" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3841,10 +3865,10 @@
       <c r="E51">
         <v>0</v>
       </c>
-      <c r="F51">
+      <c r="F51" s="3">
         <v>12748261</v>
       </c>
-      <c r="G51">
+      <c r="G51" s="3">
         <v>0</v>
       </c>
       <c r="H51">
@@ -3867,10 +3891,10 @@
       <c r="E52">
         <v>0</v>
       </c>
-      <c r="F52">
+      <c r="F52" s="3">
         <v>11330218</v>
       </c>
-      <c r="G52">
+      <c r="G52" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3890,10 +3914,10 @@
       <c r="E53">
         <v>2.4508435497476118E-6</v>
       </c>
-      <c r="F53">
+      <c r="F53" s="3">
         <v>184727530.00525001</v>
       </c>
-      <c r="G53">
+      <c r="G53" s="3">
         <v>452.73827537417549</v>
       </c>
       <c r="H53">
@@ -3916,10 +3940,10 @@
       <c r="E54">
         <v>7.4436574317583404E-7</v>
       </c>
-      <c r="F54">
+      <c r="F54" s="3">
         <v>79784042.78475</v>
       </c>
-      <c r="G54">
+      <c r="G54" s="3">
         <v>59.388508301042982</v>
       </c>
       <c r="H54">
@@ -3942,10 +3966,10 @@
       <c r="E55">
         <v>7.3578403968243425E-5</v>
       </c>
-      <c r="F55">
+      <c r="F55" s="3">
         <v>132614577.92729621</v>
       </c>
-      <c r="G55">
+      <c r="G55" s="3">
         <v>9757.5689868126956</v>
       </c>
       <c r="H55">
@@ -3968,10 +3992,10 @@
       <c r="E56">
         <v>3.4040599923819719E-6</v>
       </c>
-      <c r="F56">
+      <c r="F56" s="3">
         <v>105493361.5907038</v>
       </c>
-      <c r="G56">
+      <c r="G56" s="3">
         <v>359.10573165279988</v>
       </c>
       <c r="H56">
@@ -3994,10 +4018,10 @@
       <c r="E57">
         <v>0</v>
       </c>
-      <c r="F57">
+      <c r="F57" s="3">
         <v>156123</v>
       </c>
-      <c r="G57">
+      <c r="G57" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4017,10 +4041,10 @@
       <c r="E58">
         <v>0</v>
       </c>
-      <c r="F58">
+      <c r="F58" s="3">
         <v>438704.72200000001</v>
       </c>
-      <c r="G58">
+      <c r="G58" s="3">
         <v>0</v>
       </c>
       <c r="H58">
@@ -4043,10 +4067,10 @@
       <c r="E59">
         <v>0</v>
       </c>
-      <c r="F59">
+      <c r="F59" s="3">
         <v>640539.32499999995</v>
       </c>
-      <c r="G59">
+      <c r="G59" s="3">
         <v>0</v>
       </c>
       <c r="H59">
@@ -4069,10 +4093,10 @@
       <c r="E60">
         <v>0</v>
       </c>
-      <c r="F60">
+      <c r="F60" s="3">
         <v>79528</v>
       </c>
-      <c r="G60">
+      <c r="G60" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4092,10 +4116,10 @@
       <c r="E61">
         <v>0</v>
       </c>
-      <c r="F61">
+      <c r="F61" s="3">
         <v>619909.95116279065</v>
       </c>
-      <c r="G61">
+      <c r="G61" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4115,10 +4139,10 @@
       <c r="E62">
         <v>0</v>
       </c>
-      <c r="F62">
+      <c r="F62" s="3">
         <v>62199.4</v>
       </c>
-      <c r="G62">
+      <c r="G62" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4138,10 +4162,10 @@
       <c r="E63">
         <v>0</v>
       </c>
-      <c r="F63">
+      <c r="F63" s="3">
         <v>492005.245</v>
       </c>
-      <c r="G63">
+      <c r="G63" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4161,10 +4185,10 @@
       <c r="E64">
         <v>0</v>
       </c>
-      <c r="F64">
+      <c r="F64" s="3">
         <v>913348.23580446152</v>
       </c>
-      <c r="G64">
+      <c r="G64" s="3">
         <v>0</v>
       </c>
       <c r="H64">
@@ -4187,10 +4211,10 @@
       <c r="E65">
         <v>0</v>
       </c>
-      <c r="F65">
+      <c r="F65" s="3">
         <v>5900901.001218589</v>
       </c>
-      <c r="G65">
+      <c r="G65" s="3">
         <v>0</v>
       </c>
       <c r="H65">
@@ -4213,10 +4237,10 @@
       <c r="E66">
         <v>7.7301323708946637E-7</v>
       </c>
-      <c r="F66">
+      <c r="F66" s="3">
         <v>4739632.0318539664</v>
       </c>
-      <c r="G66">
+      <c r="G66" s="3">
         <v>3.6637982995563592</v>
       </c>
       <c r="H66">
@@ -4239,10 +4263,10 @@
       <c r="E67">
         <v>0</v>
       </c>
-      <c r="F67">
+      <c r="F67" s="3">
         <v>4326410.9030381572</v>
       </c>
-      <c r="G67">
+      <c r="G67" s="3">
         <v>0</v>
       </c>
       <c r="H67">
@@ -4265,10 +4289,10 @@
       <c r="E68">
         <v>3.2043417855721092E-7</v>
       </c>
-      <c r="F68">
+      <c r="F68" s="3">
         <v>17226.322559848741</v>
       </c>
-      <c r="G68">
+      <c r="G68" s="3">
         <v>5.519902519026682E-3</v>
       </c>
     </row>
@@ -4288,10 +4312,10 @@
       <c r="E69">
         <v>0</v>
       </c>
-      <c r="F69">
+      <c r="F69" s="3">
         <v>93717.001999999993</v>
       </c>
-      <c r="G69">
+      <c r="G69" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4311,10 +4335,10 @@
       <c r="E70">
         <v>3.8650661854473319E-7</v>
       </c>
-      <c r="F70">
+      <c r="F70" s="3">
         <v>88026.33906281479</v>
       </c>
-      <c r="G70">
+      <c r="G70" s="3">
         <v>3.4022762654040702E-2</v>
       </c>
     </row>
@@ -4334,10 +4358,10 @@
       <c r="E71">
         <v>0</v>
       </c>
-      <c r="F71">
+      <c r="F71" s="3">
         <v>27117.873653330069</v>
       </c>
-      <c r="G71">
+      <c r="G71" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4357,10 +4381,10 @@
       <c r="E72">
         <v>6.4086835711442173E-7</v>
       </c>
-      <c r="F72">
+      <c r="F72" s="3">
         <v>8190024.8600657582</v>
       </c>
-      <c r="G72">
+      <c r="G72" s="3">
         <v>5.2487277767966143</v>
       </c>
       <c r="H72">
@@ -4383,10 +4407,10 @@
       <c r="E73">
         <v>0</v>
       </c>
-      <c r="F73">
+      <c r="F73" s="3">
         <v>4353366.5807391303</v>
       </c>
-      <c r="G73">
+      <c r="G73" s="3">
         <v>0</v>
       </c>
       <c r="H73">
@@ -4409,10 +4433,10 @@
       <c r="E74">
         <v>0</v>
       </c>
-      <c r="F74">
+      <c r="F74" s="3">
         <v>10837196.79415895</v>
       </c>
-      <c r="G74">
+      <c r="G74" s="3">
         <v>0</v>
       </c>
       <c r="H74">
@@ -4435,10 +4459,10 @@
       <c r="E75">
         <v>0</v>
       </c>
-      <c r="F75">
+      <c r="F75" s="3">
         <v>2139314.2969999998</v>
       </c>
-      <c r="G75">
+      <c r="G75" s="3">
         <v>0</v>
       </c>
       <c r="H75">
@@ -4456,7 +4480,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.140625" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -4475,10 +4500,10 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -4501,10 +4526,10 @@
       <c r="E2">
         <v>0</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="3">
         <v>2300</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4524,10 +4549,10 @@
       <c r="E3">
         <v>0</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="3">
         <v>21469.262905162061</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4547,10 +4572,10 @@
       <c r="E4">
         <v>0</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="3">
         <v>753569.72512978013</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="3">
         <v>0</v>
       </c>
       <c r="H4">
@@ -4573,10 +4598,10 @@
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="3">
         <v>700962.931795649</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="3">
         <v>0</v>
       </c>
       <c r="H5">
@@ -4599,10 +4624,10 @@
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="3">
         <v>2452355.66145615</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="3">
         <v>0</v>
       </c>
       <c r="H6">
@@ -4625,10 +4650,10 @@
       <c r="E7">
         <v>0</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="3">
         <v>1761815.053452285</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="3">
         <v>0</v>
       </c>
       <c r="H7">
@@ -4651,10 +4676,10 @@
       <c r="E8">
         <v>0</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="3">
         <v>824600.54603952006</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="3">
         <v>0</v>
       </c>
       <c r="H8">
@@ -4677,10 +4702,10 @@
       <c r="E9">
         <v>0</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="3">
         <v>342935.35396048002</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="3">
         <v>0</v>
       </c>
       <c r="H9">
@@ -4703,10 +4728,10 @@
       <c r="E10">
         <v>0</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="3">
         <v>3597855.4026433248</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="3">
         <v>0</v>
       </c>
       <c r="H10">
@@ -4729,10 +4754,10 @@
       <c r="E11">
         <v>0</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="3">
         <v>371539.38865177229</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="3">
         <v>0</v>
       </c>
       <c r="H11">
@@ -4755,10 +4780,10 @@
       <c r="E12">
         <v>0</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="3">
         <v>2478138.821705427</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4778,10 +4803,10 @@
       <c r="E13">
         <v>0</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="3">
         <v>18322212.479166672</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="3">
         <v>0</v>
       </c>
       <c r="H13">
@@ -4804,10 +4829,10 @@
       <c r="E14">
         <v>0</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="3">
         <v>6774519.576923077</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="3">
         <v>0</v>
       </c>
       <c r="H14">
@@ -4830,10 +4855,10 @@
       <c r="E15">
         <v>0</v>
       </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15">
+      <c r="F15" s="3">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4853,10 +4878,10 @@
       <c r="E16">
         <v>0</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="3">
         <v>38844786.131999999</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="3">
         <v>0</v>
       </c>
       <c r="H16">
@@ -4879,10 +4904,10 @@
       <c r="E17">
         <v>0</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="3">
         <v>15722</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4902,10 +4927,10 @@
       <c r="E18">
         <v>1.836368364239625E-7</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="3">
         <v>23373052.6192853</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="3">
         <v>4.2921534405763637</v>
       </c>
       <c r="H18">
@@ -4928,10 +4953,10 @@
       <c r="E19">
         <v>1.140459242050621E-7</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="3">
         <v>117464020.329</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="3">
         <v>13.396292759263011</v>
       </c>
       <c r="H19">
@@ -4954,10 +4979,10 @@
       <c r="E20">
         <v>0</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="3">
         <v>160428</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4977,10 +5002,10 @@
       <c r="E21">
         <v>0</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="3">
         <v>22473219.009149559</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="3">
         <v>0</v>
       </c>
       <c r="H21">
@@ -5003,10 +5028,10 @@
       <c r="E22">
         <v>7.7126814006275586E-5</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="3">
         <v>36428091.839511126</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="3">
         <v>2809.5826639095012</v>
       </c>
       <c r="H22">
@@ -5029,10 +5054,10 @@
       <c r="E23">
         <v>1.791348259102799E-3</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="3">
         <v>6906618.0694853142</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="3">
         <v>12372.158255060451</v>
       </c>
       <c r="H23">
@@ -5055,10 +5080,10 @@
       <c r="E24">
         <v>8.0756148857289366E-5</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="3">
         <v>31698095.08031968</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="3">
         <v>2559.816084798807</v>
       </c>
       <c r="H24">
@@ -5081,10 +5106,10 @@
       <c r="E25">
         <v>6.8692884514512029E-4</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="3">
         <v>6413896.8770221323</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="3">
         <v>4405.890774612707</v>
       </c>
       <c r="H25">
@@ -5107,10 +5132,10 @@
       <c r="E26">
         <v>1.0944775283704231E-3</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="3">
         <v>246476.5</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="3">
         <v>269.76299052139251</v>
       </c>
     </row>
@@ -5130,10 +5155,10 @@
       <c r="E27">
         <v>1.090010807391068E-2</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="3">
         <v>107667</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="3">
         <v>1173.5819359937409</v>
       </c>
     </row>
@@ -5153,10 +5178,10 @@
       <c r="E28">
         <v>5.5523334435985628E-3</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="3">
         <v>68683.310872100425</v>
       </c>
-      <c r="G28">
+      <c r="G28" s="3">
         <v>381.35264397224</v>
       </c>
     </row>
@@ -5176,10 +5201,10 @@
       <c r="E29">
         <v>6.8692884514512029E-4</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="3">
         <v>159857</v>
       </c>
-      <c r="G29">
+      <c r="G29" s="3">
         <v>109.8103843983635</v>
       </c>
     </row>
@@ -5199,10 +5224,10 @@
       <c r="E30" s="2">
         <v>2.1118282427345699E-3</v>
       </c>
-      <c r="F30" s="2">
+      <c r="F30" s="5">
         <v>21896431.973870799</v>
       </c>
-      <c r="G30" s="2">
+      <c r="G30" s="5">
         <v>46241.503457536608</v>
       </c>
       <c r="H30" s="2">
@@ -5225,10 +5250,10 @@
       <c r="E31" s="2">
         <v>2.000886788871856E-2</v>
       </c>
-      <c r="F31" s="2">
+      <c r="F31" s="5">
         <v>25577560.136865132</v>
       </c>
-      <c r="G31" s="2">
+      <c r="G31" s="5">
         <v>511778.02169428871</v>
       </c>
       <c r="H31" s="2">
@@ -5251,10 +5276,10 @@
       <c r="E32" s="2">
         <v>5.5523334435985628E-3</v>
       </c>
-      <c r="F32" s="2">
+      <c r="F32" s="5">
         <v>29024889.379979141</v>
       </c>
-      <c r="G32" s="2">
+      <c r="G32" s="5">
         <v>161155.86400120691</v>
       </c>
       <c r="H32" s="2">
@@ -5277,10 +5302,10 @@
       <c r="E33" s="2">
         <v>2.5940985172919042E-3</v>
       </c>
-      <c r="F33" s="2">
+      <c r="F33" s="5">
         <v>33392176.301814649</v>
       </c>
-      <c r="G33" s="2">
+      <c r="G33" s="5">
         <v>86622.595033687234</v>
       </c>
       <c r="H33" s="2">
@@ -5303,10 +5328,10 @@
       <c r="E34">
         <v>0</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="3">
         <v>2017068.655317503</v>
       </c>
-      <c r="G34">
+      <c r="G34" s="3">
         <v>0</v>
       </c>
       <c r="H34">
@@ -5329,10 +5354,10 @@
       <c r="E35">
         <v>5.7883423581439412E-6</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="3">
         <v>2115740.8440453699</v>
       </c>
-      <c r="G35">
+      <c r="G35" s="3">
         <v>12.246632346443031</v>
       </c>
       <c r="H35">
@@ -5355,10 +5380,10 @@
       <c r="E36">
         <v>0</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="3">
         <v>564901.33666130423</v>
       </c>
-      <c r="G36">
+      <c r="G36" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5378,10 +5403,10 @@
       <c r="E37">
         <v>0</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="3">
         <v>152326.6300376268</v>
       </c>
-      <c r="G37">
+      <c r="G37" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5401,10 +5426,10 @@
       <c r="E38">
         <v>0</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="3">
         <v>1264097.995133939</v>
       </c>
-      <c r="G38">
+      <c r="G38" s="3">
         <v>0</v>
       </c>
       <c r="H38">
@@ -5427,10 +5452,10 @@
       <c r="E39">
         <v>0</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="3">
         <v>167204.17654073989</v>
       </c>
-      <c r="G39">
+      <c r="G39" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5450,10 +5475,10 @@
       <c r="E40">
         <v>5.9606897926980462E-4</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="3">
         <v>1519335.2860000001</v>
       </c>
-      <c r="G40">
+      <c r="G40" s="3">
         <v>905.6286330946167</v>
       </c>
       <c r="H40">
@@ -5476,10 +5501,10 @@
       <c r="E41">
         <v>2.1123728539906361E-2</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="3">
         <v>19051</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="3">
         <v>402.42815241375598</v>
       </c>
     </row>
@@ -5499,10 +5524,10 @@
       <c r="E42">
         <v>2.1123728539906361E-2</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="3">
         <v>564641.01</v>
       </c>
-      <c r="G42">
+      <c r="G42" s="3">
         <v>11927.323417738549</v>
       </c>
       <c r="H42">
@@ -5525,10 +5550,10 @@
       <c r="E43">
         <v>0</v>
       </c>
-      <c r="F43">
+      <c r="F43" s="3">
         <v>31608</v>
       </c>
-      <c r="G43">
+      <c r="G43" s="3">
         <v>0</v>
       </c>
       <c r="H43">
@@ -5551,10 +5576,10 @@
       <c r="E44">
         <v>0</v>
       </c>
-      <c r="F44">
+      <c r="F44" s="3">
         <v>202455.1253333333</v>
       </c>
-      <c r="G44">
+      <c r="G44" s="3">
         <v>0</v>
       </c>
       <c r="H44">
@@ -5577,10 +5602,10 @@
       <c r="E45">
         <v>0</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="3">
         <v>301461.19276470592</v>
       </c>
-      <c r="G45">
+      <c r="G45" s="3">
         <v>0</v>
       </c>
       <c r="H45">
@@ -5603,10 +5628,10 @@
       <c r="E46">
         <v>0</v>
       </c>
-      <c r="F46">
+      <c r="F46" s="3">
         <v>248842.38373118901</v>
       </c>
-      <c r="G46">
+      <c r="G46" s="3">
         <v>0</v>
       </c>
       <c r="H46">
@@ -5629,10 +5654,10 @@
       <c r="E47">
         <v>0</v>
       </c>
-      <c r="F47">
+      <c r="F47" s="3">
         <v>792319</v>
       </c>
-      <c r="G47">
+      <c r="G47" s="3">
         <v>0</v>
       </c>
       <c r="H47">
@@ -5655,10 +5680,10 @@
       <c r="E48">
         <v>0</v>
       </c>
-      <c r="F48">
+      <c r="F48" s="3">
         <v>1172545</v>
       </c>
-      <c r="G48">
+      <c r="G48" s="3">
         <v>0</v>
       </c>
       <c r="H48">
@@ -5681,10 +5706,10 @@
       <c r="E49">
         <v>0</v>
       </c>
-      <c r="F49">
+      <c r="F49" s="3">
         <v>1892795</v>
       </c>
-      <c r="G49">
+      <c r="G49" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5704,10 +5729,10 @@
       <c r="E50">
         <v>0</v>
       </c>
-      <c r="F50">
+      <c r="F50" s="3">
         <v>20798650</v>
       </c>
-      <c r="G50">
+      <c r="G50" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5727,10 +5752,10 @@
       <c r="E51">
         <v>0</v>
       </c>
-      <c r="F51">
+      <c r="F51" s="3">
         <v>12748261</v>
       </c>
-      <c r="G51">
+      <c r="G51" s="3">
         <v>0</v>
       </c>
       <c r="H51">
@@ -5753,10 +5778,10 @@
       <c r="E52">
         <v>0</v>
       </c>
-      <c r="F52">
+      <c r="F52" s="3">
         <v>11330218</v>
       </c>
-      <c r="G52">
+      <c r="G52" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5776,10 +5801,10 @@
       <c r="E53">
         <v>1.016309478451792E-4</v>
       </c>
-      <c r="F53">
+      <c r="F53" s="3">
         <v>184727530.00525001</v>
       </c>
-      <c r="G53">
+      <c r="G53" s="3">
         <v>18774.033967532341</v>
       </c>
       <c r="H53">
@@ -5802,10 +5827,10 @@
       <c r="E54">
         <v>3.0292449374460031E-5</v>
       </c>
-      <c r="F54">
+      <c r="F54" s="3">
         <v>79784042.78475</v>
       </c>
-      <c r="G54">
+      <c r="G54" s="3">
         <v>2416.8540769467918</v>
       </c>
       <c r="H54">
@@ -5828,10 +5853,10 @@
       <c r="E55">
         <v>6.4968500717780322E-6</v>
       </c>
-      <c r="F55">
+      <c r="F55" s="3">
         <v>132614577.92729621</v>
       </c>
-      <c r="G55">
+      <c r="G55" s="3">
         <v>861.57703012576758</v>
       </c>
       <c r="H55">
@@ -5854,10 +5879,10 @@
       <c r="E56">
         <v>4.0563463484641052E-5</v>
       </c>
-      <c r="F56">
+      <c r="F56" s="3">
         <v>105493361.5907038</v>
       </c>
-      <c r="G56">
+      <c r="G56" s="3">
         <v>4279.1761207565496</v>
       </c>
       <c r="H56">
@@ -5880,10 +5905,10 @@
       <c r="E57">
         <v>0</v>
       </c>
-      <c r="F57">
+      <c r="F57" s="3">
         <v>156123</v>
       </c>
-      <c r="G57">
+      <c r="G57" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5903,10 +5928,10 @@
       <c r="E58">
         <v>0</v>
       </c>
-      <c r="F58">
+      <c r="F58" s="3">
         <v>438704.72200000001</v>
       </c>
-      <c r="G58">
+      <c r="G58" s="3">
         <v>0</v>
       </c>
       <c r="H58">
@@ -5929,10 +5954,10 @@
       <c r="E59">
         <v>6.6502380884435052E-6</v>
       </c>
-      <c r="F59">
+      <c r="F59" s="3">
         <v>640539.32499999995</v>
       </c>
-      <c r="G59">
+      <c r="G59" s="3">
         <v>4.2597390162608928</v>
       </c>
       <c r="H59">
@@ -5955,10 +5980,10 @@
       <c r="E60">
         <v>0</v>
       </c>
-      <c r="F60">
+      <c r="F60" s="3">
         <v>79528</v>
       </c>
-      <c r="G60">
+      <c r="G60" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5978,10 +6003,10 @@
       <c r="E61">
         <v>0</v>
       </c>
-      <c r="F61">
+      <c r="F61" s="3">
         <v>619909.95116279065</v>
       </c>
-      <c r="G61">
+      <c r="G61" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6001,10 +6026,10 @@
       <c r="E62">
         <v>0</v>
       </c>
-      <c r="F62">
+      <c r="F62" s="3">
         <v>62199.4</v>
       </c>
-      <c r="G62">
+      <c r="G62" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6024,10 +6049,10 @@
       <c r="E63">
         <v>0</v>
       </c>
-      <c r="F63">
+      <c r="F63" s="3">
         <v>492005.245</v>
       </c>
-      <c r="G63">
+      <c r="G63" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6047,10 +6072,10 @@
       <c r="E64">
         <v>0</v>
       </c>
-      <c r="F64">
+      <c r="F64" s="3">
         <v>913348.23580446152</v>
       </c>
-      <c r="G64">
+      <c r="G64" s="3">
         <v>0</v>
       </c>
       <c r="H64">
@@ -6073,10 +6098,10 @@
       <c r="E65">
         <v>0</v>
       </c>
-      <c r="F65">
+      <c r="F65" s="3">
         <v>5900901.001218589</v>
       </c>
-      <c r="G65">
+      <c r="G65" s="3">
         <v>0</v>
       </c>
       <c r="H65">
@@ -6099,10 +6124,10 @@
       <c r="E66">
         <v>1.5151059446953541E-5</v>
       </c>
-      <c r="F66">
+      <c r="F66" s="3">
         <v>4739632.0318539664</v>
       </c>
-      <c r="G66">
+      <c r="G66" s="3">
         <v>71.810446671304646</v>
       </c>
       <c r="H66">
@@ -6125,10 +6150,10 @@
       <c r="E67">
         <v>2.6667609846691722E-5</v>
       </c>
-      <c r="F67">
+      <c r="F67" s="3">
         <v>4326410.9030381572</v>
       </c>
-      <c r="G67">
+      <c r="G67" s="3">
         <v>115.37503799869479</v>
       </c>
       <c r="H67">
@@ -6151,10 +6176,10 @@
       <c r="E68">
         <v>1.0681139285240361E-6</v>
       </c>
-      <c r="F68">
+      <c r="F68" s="3">
         <v>17226.322559848741</v>
       </c>
-      <c r="G68">
+      <c r="G68" s="3">
         <v>1.8399675063422279E-2</v>
       </c>
     </row>
@@ -6174,10 +6199,10 @@
       <c r="E69">
         <v>0</v>
       </c>
-      <c r="F69">
+      <c r="F69" s="3">
         <v>93717.001999999993</v>
       </c>
-      <c r="G69">
+      <c r="G69" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6197,10 +6222,10 @@
       <c r="E70">
         <v>2.4106733648042219E-5</v>
       </c>
-      <c r="F70">
+      <c r="F70" s="3">
         <v>88026.33906281479</v>
       </c>
-      <c r="G70">
+      <c r="G70" s="3">
         <v>2.1220275097995311</v>
       </c>
     </row>
@@ -6220,10 +6245,10 @@
       <c r="E71">
         <v>1.7175976198785941E-5</v>
       </c>
-      <c r="F71">
+      <c r="F71" s="3">
         <v>27117.873653330069</v>
       </c>
-      <c r="G71">
+      <c r="G71" s="3">
         <v>0.46577595243128161</v>
       </c>
     </row>
@@ -6243,10 +6268,10 @@
       <c r="E72">
         <v>2.1362278570480731E-6</v>
       </c>
-      <c r="F72">
+      <c r="F72" s="3">
         <v>8190024.8600657582</v>
       </c>
-      <c r="G72">
+      <c r="G72" s="3">
         <v>17.49575925598872</v>
       </c>
       <c r="H72">
@@ -6269,10 +6294,10 @@
       <c r="E73">
         <v>0</v>
       </c>
-      <c r="F73">
+      <c r="F73" s="3">
         <v>4353366.5807391303</v>
       </c>
-      <c r="G73">
+      <c r="G73" s="3">
         <v>0</v>
       </c>
       <c r="H73">
@@ -6295,10 +6320,10 @@
       <c r="E74">
         <v>3.3062407849130902E-5</v>
       </c>
-      <c r="F74">
+      <c r="F74" s="3">
         <v>10837196.79415895</v>
       </c>
-      <c r="G74">
+      <c r="G74" s="3">
         <v>358.30382034977703</v>
       </c>
       <c r="H74">
@@ -6321,10 +6346,10 @@
       <c r="E75">
         <v>7.6843425508801645E-6</v>
       </c>
-      <c r="F75">
+      <c r="F75" s="3">
         <v>2139314.2969999998</v>
       </c>
-      <c r="G75">
+      <c r="G75" s="3">
         <v>16.439223882143381</v>
       </c>
       <c r="H75">
@@ -6340,6 +6365,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="15.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -6357,10 +6386,10 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -6383,10 +6412,10 @@
       <c r="E2">
         <v>0</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="3">
         <v>2300</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6406,10 +6435,10 @@
       <c r="E3">
         <v>0</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="3">
         <v>21469.262905162061</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6429,10 +6458,10 @@
       <c r="E4">
         <v>0</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="3">
         <v>753569.72512978013</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="3">
         <v>0</v>
       </c>
       <c r="H4">
@@ -6455,10 +6484,10 @@
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="3">
         <v>700962.931795649</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="3">
         <v>0</v>
       </c>
       <c r="H5">
@@ -6481,10 +6510,10 @@
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="3">
         <v>2452355.66145615</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="3">
         <v>0</v>
       </c>
       <c r="H6">
@@ -6507,10 +6536,10 @@
       <c r="E7">
         <v>0</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="3">
         <v>1761815.053452285</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="3">
         <v>0</v>
       </c>
       <c r="H7">
@@ -6533,10 +6562,10 @@
       <c r="E8">
         <v>0</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="3">
         <v>824600.54603952006</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="3">
         <v>0</v>
       </c>
       <c r="H8">
@@ -6559,10 +6588,10 @@
       <c r="E9">
         <v>0</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="3">
         <v>342935.35396048002</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="3">
         <v>0</v>
       </c>
       <c r="H9">
@@ -6585,10 +6614,10 @@
       <c r="E10">
         <v>0</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="3">
         <v>3597855.4026433248</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="3">
         <v>0</v>
       </c>
       <c r="H10">
@@ -6611,10 +6640,10 @@
       <c r="E11">
         <v>0</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="3">
         <v>371539.38865177229</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="3">
         <v>0</v>
       </c>
       <c r="H11">
@@ -6637,10 +6666,10 @@
       <c r="E12">
         <v>0</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="3">
         <v>2478138.821705427</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6660,10 +6689,10 @@
       <c r="E13">
         <v>0</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="3">
         <v>18322212.479166672</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="3">
         <v>0</v>
       </c>
       <c r="H13">
@@ -6686,10 +6715,10 @@
       <c r="E14">
         <v>0</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="3">
         <v>6774519.576923077</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="3">
         <v>0</v>
       </c>
       <c r="H14">
@@ -6712,10 +6741,10 @@
       <c r="E15">
         <v>0</v>
       </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15">
+      <c r="F15" s="3">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6735,10 +6764,10 @@
       <c r="E16">
         <v>0</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="3">
         <v>38844786.131999999</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="3">
         <v>0</v>
       </c>
       <c r="H16">
@@ -6761,10 +6790,10 @@
       <c r="E17">
         <v>0</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="3">
         <v>15722</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6784,10 +6813,10 @@
       <c r="E18">
         <v>0</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="3">
         <v>23373052.6192853</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="3">
         <v>0</v>
       </c>
       <c r="H18">
@@ -6810,10 +6839,10 @@
       <c r="E19">
         <v>0</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="3">
         <v>117464020.329</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="3">
         <v>0</v>
       </c>
       <c r="H19">
@@ -6836,10 +6865,10 @@
       <c r="E20">
         <v>0</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="3">
         <v>160428</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6859,10 +6888,10 @@
       <c r="E21">
         <v>0</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="3">
         <v>22473219.009149559</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="3">
         <v>0</v>
       </c>
       <c r="H21">
@@ -6885,10 +6914,10 @@
       <c r="E22">
         <v>6.9010075675589755E-5</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="3">
         <v>36428091.839511126</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="3">
         <v>2513.9053745619972</v>
       </c>
       <c r="H22">
@@ -6911,10 +6940,10 @@
       <c r="E23">
         <v>3.4115193104255872E-3</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="3">
         <v>6906618.0694853142</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="3">
         <v>23562.06091378344</v>
       </c>
       <c r="H23">
@@ -6937,10 +6966,10 @@
       <c r="E24">
         <v>2.0867652178946651E-4</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="3">
         <v>31698095.08031968</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="3">
         <v>6614.6482287129093</v>
       </c>
       <c r="H24">
@@ -6963,10 +6992,10 @@
       <c r="E25">
         <v>2.4188189942729401E-3</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="3">
         <v>6413896.8770221323</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="3">
         <v>15514.055593449029</v>
       </c>
       <c r="H25">
@@ -6989,10 +7018,10 @@
       <c r="E26">
         <v>7.95277733578326E-3</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="3">
         <v>246476.5</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="3">
         <v>1960.1727230031829</v>
       </c>
     </row>
@@ -7012,10 +7041,10 @@
       <c r="E27">
         <v>1.7456413613458271E-2</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="3">
         <v>107667</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="3">
         <v>1879.479684520212</v>
       </c>
     </row>
@@ -7035,10 +7064,10 @@
       <c r="E28">
         <v>3.9856207982979348E-2</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="3">
         <v>68683.310872100425</v>
       </c>
-      <c r="G28">
+      <c r="G28" s="3">
         <v>2737.4563230780609</v>
       </c>
     </row>
@@ -7058,10 +7087,10 @@
       <c r="E29">
         <v>2.4188189942729401E-3</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="3">
         <v>159857</v>
       </c>
-      <c r="G29">
+      <c r="G29" s="3">
         <v>386.66514796748942</v>
       </c>
     </row>
@@ -7081,10 +7110,10 @@
       <c r="E30">
         <v>1.5836544595890931E-2</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="3">
         <v>21896431.973870799</v>
       </c>
-      <c r="G30">
+      <c r="G30" s="3">
         <v>346763.82144509692</v>
       </c>
       <c r="H30">
@@ -7107,10 +7136,10 @@
       <c r="E31">
         <v>3.1501307916490959E-2</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="3">
         <v>25577560.136865132</v>
       </c>
-      <c r="G31">
+      <c r="G31" s="3">
         <v>805726.59762395313</v>
       </c>
       <c r="H31">
@@ -7133,10 +7162,10 @@
       <c r="E32">
         <v>3.9856207982979348E-2</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="3">
         <v>29024889.379979141</v>
       </c>
-      <c r="G32">
+      <c r="G32" s="3">
         <v>1156822.0278114169</v>
       </c>
       <c r="H32">
@@ -7159,10 +7188,10 @@
       <c r="E33">
         <v>1.9483804256839439E-2</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="3">
         <v>33392176.301814649</v>
       </c>
-      <c r="G33">
+      <c r="G33" s="3">
         <v>650606.62677442911</v>
       </c>
       <c r="H33">
@@ -7185,10 +7214,10 @@
       <c r="E34">
         <v>3.8871022846653247E-6</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="3">
         <v>2017068.655317503</v>
       </c>
-      <c r="G34">
+      <c r="G34" s="3">
         <v>7.8405521784114809</v>
       </c>
       <c r="H34">
@@ -7211,10 +7240,10 @@
       <c r="E35">
         <v>5.7202442127540117E-5</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="3">
         <v>2115740.8440453699</v>
       </c>
-      <c r="G35">
+      <c r="G35" s="3">
         <v>121.02554318837819</v>
       </c>
       <c r="H35">
@@ -7237,10 +7266,10 @@
       <c r="E36">
         <v>0</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="3">
         <v>564901.33666130423</v>
       </c>
-      <c r="G36">
+      <c r="G36" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7260,10 +7289,10 @@
       <c r="E37">
         <v>0</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="3">
         <v>152326.6300376268</v>
       </c>
-      <c r="G37">
+      <c r="G37" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7283,10 +7312,10 @@
       <c r="E38">
         <v>0</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="3">
         <v>1264097.995133939</v>
       </c>
-      <c r="G38">
+      <c r="G38" s="3">
         <v>0</v>
       </c>
       <c r="H38">
@@ -7309,10 +7338,10 @@
       <c r="E39">
         <v>0</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="3">
         <v>167204.17654073989</v>
       </c>
-      <c r="G39">
+      <c r="G39" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7332,10 +7361,10 @@
       <c r="E40">
         <v>6.9119918000175324E-3</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="3">
         <v>1519335.2860000001</v>
       </c>
-      <c r="G40">
+      <c r="G40" s="3">
         <v>10501.63303830929</v>
       </c>
       <c r="H40">
@@ -7358,10 +7387,10 @@
       <c r="E41">
         <v>0</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="3">
         <v>19051</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7381,10 +7410,10 @@
       <c r="E42">
         <v>0</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="3">
         <v>564641.01</v>
       </c>
-      <c r="G42">
+      <c r="G42" s="3">
         <v>0</v>
       </c>
       <c r="H42">
@@ -7407,10 +7436,10 @@
       <c r="E43">
         <v>0</v>
       </c>
-      <c r="F43">
+      <c r="F43" s="3">
         <v>31608</v>
       </c>
-      <c r="G43">
+      <c r="G43" s="3">
         <v>0</v>
       </c>
       <c r="H43">
@@ -7433,10 +7462,10 @@
       <c r="E44">
         <v>0</v>
       </c>
-      <c r="F44">
+      <c r="F44" s="3">
         <v>202455.1253333333</v>
       </c>
-      <c r="G44">
+      <c r="G44" s="3">
         <v>0</v>
       </c>
       <c r="H44">
@@ -7459,10 +7488,10 @@
       <c r="E45">
         <v>0</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="3">
         <v>301461.19276470592</v>
       </c>
-      <c r="G45">
+      <c r="G45" s="3">
         <v>0</v>
       </c>
       <c r="H45">
@@ -7485,10 +7514,10 @@
       <c r="E46">
         <v>0</v>
       </c>
-      <c r="F46">
+      <c r="F46" s="3">
         <v>248842.38373118901</v>
       </c>
-      <c r="G46">
+      <c r="G46" s="3">
         <v>0</v>
       </c>
       <c r="H46">
@@ -7511,10 +7540,10 @@
       <c r="E47">
         <v>0</v>
       </c>
-      <c r="F47">
+      <c r="F47" s="3">
         <v>792319</v>
       </c>
-      <c r="G47">
+      <c r="G47" s="3">
         <v>0</v>
       </c>
       <c r="H47">
@@ -7537,10 +7566,10 @@
       <c r="E48">
         <v>0</v>
       </c>
-      <c r="F48">
+      <c r="F48" s="3">
         <v>1172545</v>
       </c>
-      <c r="G48">
+      <c r="G48" s="3">
         <v>0</v>
       </c>
       <c r="H48">
@@ -7563,10 +7592,10 @@
       <c r="E49">
         <v>0</v>
       </c>
-      <c r="F49">
+      <c r="F49" s="3">
         <v>1892795</v>
       </c>
-      <c r="G49">
+      <c r="G49" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7586,10 +7615,10 @@
       <c r="E50">
         <v>0</v>
       </c>
-      <c r="F50">
+      <c r="F50" s="3">
         <v>20798650</v>
       </c>
-      <c r="G50">
+      <c r="G50" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7609,10 +7638,10 @@
       <c r="E51">
         <v>0</v>
       </c>
-      <c r="F51">
+      <c r="F51" s="3">
         <v>12748261</v>
       </c>
-      <c r="G51">
+      <c r="G51" s="3">
         <v>0</v>
       </c>
       <c r="H51">
@@ -7635,10 +7664,10 @@
       <c r="E52">
         <v>0</v>
       </c>
-      <c r="F52">
+      <c r="F52" s="3">
         <v>11330218</v>
       </c>
-      <c r="G52">
+      <c r="G52" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7658,10 +7687,10 @@
       <c r="E53">
         <v>1.8776623969840581E-7</v>
       </c>
-      <c r="F53">
+      <c r="F53" s="3">
         <v>184727530.00525001</v>
       </c>
-      <c r="G53">
+      <c r="G53" s="3">
         <v>34.685593677860211</v>
       </c>
       <c r="H53">
@@ -7684,10 +7713,10 @@
       <c r="E54">
         <v>2.5890982371333359E-7</v>
       </c>
-      <c r="F54">
+      <c r="F54" s="3">
         <v>79784042.78475</v>
       </c>
-      <c r="G54">
+      <c r="G54" s="3">
         <v>20.656872452536689</v>
       </c>
       <c r="H54">
@@ -7710,10 +7739,10 @@
       <c r="E55">
         <v>1.0407575357702671E-6</v>
       </c>
-      <c r="F55">
+      <c r="F55" s="3">
         <v>132614577.92729621</v>
       </c>
-      <c r="G55">
+      <c r="G55" s="3">
         <v>138.01962133082679</v>
       </c>
       <c r="H55">
@@ -7736,10 +7765,10 @@
       <c r="E56">
         <v>1.9017094929508229E-8</v>
       </c>
-      <c r="F56">
+      <c r="F56" s="3">
         <v>105493361.5907038</v>
       </c>
-      <c r="G56">
+      <c r="G56" s="3">
         <v>2.0061772718033519</v>
       </c>
       <c r="H56">
@@ -7762,10 +7791,10 @@
       <c r="E57">
         <v>0</v>
       </c>
-      <c r="F57">
+      <c r="F57" s="3">
         <v>156123</v>
       </c>
-      <c r="G57">
+      <c r="G57" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7785,10 +7814,10 @@
       <c r="E58">
         <v>0</v>
       </c>
-      <c r="F58">
+      <c r="F58" s="3">
         <v>438704.72200000001</v>
       </c>
-      <c r="G58">
+      <c r="G58" s="3">
         <v>0</v>
       </c>
       <c r="H58">
@@ -7811,10 +7840,10 @@
       <c r="E59">
         <v>2.216746029481168E-6</v>
       </c>
-      <c r="F59">
+      <c r="F59" s="3">
         <v>640539.32499999995</v>
       </c>
-      <c r="G59">
+      <c r="G59" s="3">
         <v>1.419913005420298</v>
       </c>
       <c r="H59">
@@ -7837,10 +7866,10 @@
       <c r="E60">
         <v>0</v>
       </c>
-      <c r="F60">
+      <c r="F60" s="3">
         <v>79528</v>
       </c>
-      <c r="G60">
+      <c r="G60" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7860,10 +7889,10 @@
       <c r="E61">
         <v>0</v>
       </c>
-      <c r="F61">
+      <c r="F61" s="3">
         <v>619909.95116279065</v>
       </c>
-      <c r="G61">
+      <c r="G61" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7883,10 +7912,10 @@
       <c r="E62">
         <v>0</v>
       </c>
-      <c r="F62">
+      <c r="F62" s="3">
         <v>62199.4</v>
       </c>
-      <c r="G62">
+      <c r="G62" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7906,10 +7935,10 @@
       <c r="E63">
         <v>0</v>
       </c>
-      <c r="F63">
+      <c r="F63" s="3">
         <v>492005.245</v>
       </c>
-      <c r="G63">
+      <c r="G63" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7929,10 +7958,10 @@
       <c r="E64">
         <v>0</v>
       </c>
-      <c r="F64">
+      <c r="F64" s="3">
         <v>913348.23580446152</v>
       </c>
-      <c r="G64">
+      <c r="G64" s="3">
         <v>0</v>
       </c>
       <c r="H64">
@@ -7955,10 +7984,10 @@
       <c r="E65">
         <v>3.1268862527593631E-6</v>
       </c>
-      <c r="F65">
+      <c r="F65" s="3">
         <v>5900901.001218589</v>
       </c>
-      <c r="G65">
+      <c r="G65" s="3">
         <v>18.451446219604371</v>
       </c>
       <c r="H65">
@@ -7981,10 +8010,10 @@
       <c r="E66">
         <v>6.3387085441336233E-6</v>
       </c>
-      <c r="F66">
+      <c r="F66" s="3">
         <v>4739632.0318539664</v>
       </c>
-      <c r="G66">
+      <c r="G66" s="3">
         <v>30.04314605636214</v>
       </c>
       <c r="H66">
@@ -8007,10 +8036,10 @@
       <c r="E67">
         <v>1.6000565908015041E-6</v>
       </c>
-      <c r="F67">
+      <c r="F67" s="3">
         <v>4326410.9030381572</v>
       </c>
-      <c r="G67">
+      <c r="G67" s="3">
         <v>6.9225022799216882</v>
       </c>
       <c r="H67">
@@ -8033,10 +8062,10 @@
       <c r="E68">
         <v>5.3405696426201816E-7</v>
       </c>
-      <c r="F68">
+      <c r="F68" s="3">
         <v>17226.322559848741</v>
       </c>
-      <c r="G68">
+      <c r="G68" s="3">
         <v>9.1998375317111376E-3</v>
       </c>
     </row>
@@ -8056,10 +8085,10 @@
       <c r="E69">
         <v>1.563443126379682E-6</v>
       </c>
-      <c r="F69">
+      <c r="F69" s="3">
         <v>93717.001999999993</v>
       </c>
-      <c r="G69">
+      <c r="G69" s="3">
         <v>0.1465212026018109</v>
       </c>
     </row>
@@ -8079,10 +8108,10 @@
       <c r="E70">
         <v>3.1693542720668121E-6</v>
       </c>
-      <c r="F70">
+      <c r="F70" s="3">
         <v>88026.33906281479</v>
       </c>
-      <c r="G70">
+      <c r="G70" s="3">
         <v>0.2789866537631337</v>
       </c>
     </row>
@@ -8102,10 +8131,10 @@
       <c r="E71">
         <v>8.0002829540075183E-7</v>
       </c>
-      <c r="F71">
+      <c r="F71" s="3">
         <v>27117.873653330069</v>
       </c>
-      <c r="G71">
+      <c r="G71" s="3">
         <v>2.1695066233766609E-2</v>
       </c>
     </row>
@@ -8125,10 +8154,10 @@
       <c r="E72">
         <v>1.0681139285240361E-6</v>
       </c>
-      <c r="F72">
+      <c r="F72" s="3">
         <v>8190024.8600657582</v>
       </c>
-      <c r="G72">
+      <c r="G72" s="3">
         <v>8.747879627994358</v>
       </c>
       <c r="H72">
@@ -8151,10 +8180,10 @@
       <c r="E73">
         <v>0</v>
       </c>
-      <c r="F73">
+      <c r="F73" s="3">
         <v>4353366.5807391303</v>
       </c>
-      <c r="G73">
+      <c r="G73" s="3">
         <v>0</v>
       </c>
       <c r="H73">
@@ -8177,10 +8206,10 @@
       <c r="E74">
         <v>0</v>
       </c>
-      <c r="F74">
+      <c r="F74" s="3">
         <v>10837196.79415895</v>
       </c>
-      <c r="G74">
+      <c r="G74" s="3">
         <v>0</v>
       </c>
       <c r="H74">
@@ -8203,10 +8232,10 @@
       <c r="E75">
         <v>0</v>
       </c>
-      <c r="F75">
+      <c r="F75" s="3">
         <v>2139314.2969999998</v>
       </c>
-      <c r="G75">
+      <c r="G75" s="3">
         <v>0</v>
       </c>
       <c r="H75">
@@ -8287,6 +8316,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -8312,19 +8348,19 @@
       <c r="A2" t="s">
         <v>85</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="3">
         <v>7426545</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="3">
         <v>137813</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="3">
         <v>3025979</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="3">
         <v>10590337</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="3">
         <v>4803.696062957024</v>
       </c>
     </row>
@@ -8332,19 +8368,19 @@
       <c r="A3" t="s">
         <v>86</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3">
         <v>11031839</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="3">
         <v>95068</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="3">
         <v>490416</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="3">
         <v>11617323</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="3">
         <v>5269.5290770444872</v>
       </c>
     </row>
@@ -8352,19 +8388,19 @@
       <c r="A4" t="s">
         <v>87</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3">
         <v>27279750</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="3">
         <v>186489</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="3">
         <v>870063</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="3">
         <v>28336302</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="3">
         <v>12853.130391994249</v>
       </c>
     </row>
@@ -8372,19 +8408,19 @@
       <c r="A5" t="s">
         <v>88</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <v>59884972</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="3">
         <v>285</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="3">
         <v>2715331</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="3">
         <v>62600588</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="3">
         <v>28395.149098125468</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add my Rproj back in and some other files
</commit_message>
<xml_diff>
--- a/CAMS/SMB_FY2019_discRd_BG_example.xlsx
+++ b/CAMS/SMB_FY2019_discRd_BG_example.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="12" windowWidth="16092" windowHeight="9660" activeTab="7"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="mack" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="catch" sheetId="5" r:id="rId5"/>
     <sheet name="summary" sheetId="6" r:id="rId6"/>
     <sheet name="Sheet1" sheetId="7" r:id="rId7"/>
-    <sheet name="Sheet2" sheetId="8" r:id="rId8"/>
+    <sheet name="ACL CAMS compare" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
@@ -717,15 +717,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M75"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -751,7 +751,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -774,7 +774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -797,7 +797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -823,7 +823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -849,7 +849,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -875,7 +875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -901,7 +901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -927,7 +927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -953,7 +953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -979,7 +979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>6.6287993710171964</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1054,7 +1054,7 @@
         <v>0.43</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -1080,7 +1080,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -1103,7 +1103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1129,7 +1129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -1178,7 +1178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -1227,7 +1227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -1253,7 +1253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -1291,7 +1291,7 @@
         <v>81446701.866338253</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -1317,7 +1317,7 @@
         <v>0.48</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -1343,7 +1343,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -1369,7 +1369,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>32</v>
       </c>
@@ -1392,7 +1392,7 @@
         <v>1824.7154300329271</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>33</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>223.75221846819571</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>110.2248865819265</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>35</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>10.88872554504216</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>36</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>109891057.79252972</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>37</v>
       </c>
@@ -1525,7 +1525,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>38</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>0.73</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>39</v>
       </c>
@@ -1577,7 +1577,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>40</v>
       </c>
@@ -1603,7 +1603,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>41</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>4299</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -1679,7 +1679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>44</v>
       </c>
@@ -1705,7 +1705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>45</v>
       </c>
@@ -1728,7 +1728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>46</v>
       </c>
@@ -1754,7 +1754,7 @@
         <v>0.48</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>47</v>
       </c>
@@ -1777,7 +1777,7 @@
         <v>0.51264732791561285</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>48</v>
       </c>
@@ -1803,7 +1803,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>49</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>50</v>
       </c>
@@ -1855,7 +1855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>51</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>52</v>
       </c>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>53</v>
       </c>
@@ -1933,7 +1933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>54</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>55</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>56</v>
       </c>
@@ -2005,7 +2005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>57</v>
       </c>
@@ -2031,7 +2031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>58</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>59</v>
       </c>
@@ -2080,7 +2080,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>60</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>0.77</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>61</v>
       </c>
@@ -2132,7 +2132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>62</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>63</v>
       </c>
@@ -2181,7 +2181,7 @@
         <v>3.8994014388944409</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>64</v>
       </c>
@@ -2207,7 +2207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>65</v>
       </c>
@@ -2233,7 +2233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>66</v>
       </c>
@@ -2256,7 +2256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>67</v>
       </c>
@@ -2279,7 +2279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>68</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>69</v>
       </c>
@@ -2325,7 +2325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>70</v>
       </c>
@@ -2351,7 +2351,7 @@
         <v>0.59</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>71</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>72</v>
       </c>
@@ -2403,7 +2403,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>73</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>0.56999999999999995</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>74</v>
       </c>
@@ -2452,7 +2452,7 @@
         <v>23.56468386024325</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>75</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>5.1088032127543244</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>76</v>
       </c>
@@ -2498,7 +2498,7 @@
         <v>10.96258570208175</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>77</v>
       </c>
@@ -2521,7 +2521,7 @@
         <v>9.40119536796553E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>78</v>
       </c>
@@ -2547,7 +2547,7 @@
         <v>0.61</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>79</v>
       </c>
@@ -2573,7 +2573,7 @@
         <v>0.68</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>80</v>
       </c>
@@ -2599,7 +2599,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>81</v>
       </c>
@@ -2633,14 +2633,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H75"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="6" max="6" width="15.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2666,7 +2666,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2712,7 +2712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -2738,7 +2738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -2790,7 +2790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -2842,7 +2842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -2868,7 +2868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2894,7 +2894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -2920,7 +2920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -2943,7 +2943,7 @@
         <v>9.7482343691429367</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -2969,7 +2969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -2995,7 +2995,7 @@
         <v>0.83</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -3018,7 +3018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -3044,7 +3044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -3067,7 +3067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -3093,7 +3093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -3119,7 +3119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -3142,7 +3142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -3168,7 +3168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -3194,7 +3194,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -3220,7 +3220,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -3246,7 +3246,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -3272,7 +3272,7 @@
         <v>0.63</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>32</v>
       </c>
@@ -3295,7 +3295,7 @@
         <v>1268.7146403800959</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>33</v>
       </c>
@@ -3318,7 +3318,7 @@
         <v>3465.0059578611422</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -3341,7 +3341,7 @@
         <v>368.28223164100888</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>35</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>15.294568251128579</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>36</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>37</v>
       </c>
@@ -3416,7 +3416,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>38</v>
       </c>
@@ -3442,7 +3442,7 @@
         <v>0.68</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>39</v>
       </c>
@@ -3468,7 +3468,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>40</v>
       </c>
@@ -3494,7 +3494,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>41</v>
       </c>
@@ -3520,7 +3520,7 @@
         <v>0.41</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -3543,7 +3543,7 @@
         <v>36521.08572088433</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -3566,7 +3566,7 @@
         <v>9847.9744198464668</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>44</v>
       </c>
@@ -3589,7 +3589,7 @@
         <v>81724.414944276039</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>45</v>
       </c>
@@ -3612,7 +3612,7 @@
         <v>10809.813445344131</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>46</v>
       </c>
@@ -3638,7 +3638,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>47</v>
       </c>
@@ -3661,7 +3661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>48</v>
       </c>
@@ -3687,7 +3687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>49</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>50</v>
       </c>
@@ -3739,7 +3739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>51</v>
       </c>
@@ -3765,7 +3765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>52</v>
       </c>
@@ -3791,7 +3791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>53</v>
       </c>
@@ -3817,7 +3817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>54</v>
       </c>
@@ -3843,7 +3843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>55</v>
       </c>
@@ -3866,7 +3866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>56</v>
       </c>
@@ -3889,7 +3889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>57</v>
       </c>
@@ -3915,7 +3915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>58</v>
       </c>
@@ -3938,7 +3938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>59</v>
       </c>
@@ -3964,7 +3964,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>60</v>
       </c>
@@ -3990,7 +3990,7 @@
         <v>0.72</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>61</v>
       </c>
@@ -4016,7 +4016,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>62</v>
       </c>
@@ -4042,7 +4042,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>63</v>
       </c>
@@ -4065,7 +4065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>64</v>
       </c>
@@ -4091,7 +4091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>65</v>
       </c>
@@ -4117,7 +4117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>66</v>
       </c>
@@ -4140,7 +4140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>67</v>
       </c>
@@ -4163,7 +4163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>68</v>
       </c>
@@ -4186,7 +4186,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>69</v>
       </c>
@@ -4209,7 +4209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>70</v>
       </c>
@@ -4235,7 +4235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>71</v>
       </c>
@@ -4261,7 +4261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>72</v>
       </c>
@@ -4287,7 +4287,7 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>73</v>
       </c>
@@ -4313,7 +4313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>74</v>
       </c>
@@ -4336,7 +4336,7 @@
         <v>5.519902519026682E-3</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>75</v>
       </c>
@@ -4359,7 +4359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>76</v>
       </c>
@@ -4382,7 +4382,7 @@
         <v>3.4022762654040702E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>77</v>
       </c>
@@ -4405,7 +4405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>78</v>
       </c>
@@ -4431,7 +4431,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>79</v>
       </c>
@@ -4457,7 +4457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>80</v>
       </c>
@@ -4483,7 +4483,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>81</v>
       </c>
@@ -4517,14 +4517,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H75"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="12.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4550,7 +4550,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4573,7 +4573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -4596,7 +4596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -4622,7 +4622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -4648,7 +4648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -4674,7 +4674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -4700,7 +4700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -4726,7 +4726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -4752,7 +4752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -4778,7 +4778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -4804,7 +4804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -4827,7 +4827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -4853,7 +4853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -4879,7 +4879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -4902,7 +4902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -4928,7 +4928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -4951,7 +4951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -4977,7 +4977,7 @@
         <v>1.06</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -5003,7 +5003,7 @@
         <v>1.1299999999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -5026,7 +5026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -5052,7 +5052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -5078,7 +5078,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -5104,7 +5104,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -5130,7 +5130,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -5156,7 +5156,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>32</v>
       </c>
@@ -5179,7 +5179,7 @@
         <v>269.76299052139251</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>33</v>
       </c>
@@ -5202,7 +5202,7 @@
         <v>1173.5819359937409</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -5225,7 +5225,7 @@
         <v>381.35264397224</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>35</v>
       </c>
@@ -5248,7 +5248,7 @@
         <v>109.8103843983635</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>36</v>
       </c>
@@ -5274,7 +5274,7 @@
         <v>0.41</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>37</v>
       </c>
@@ -5300,7 +5300,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>38</v>
       </c>
@@ -5326,7 +5326,7 @@
         <v>0.48</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>39</v>
       </c>
@@ -5352,7 +5352,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>40</v>
       </c>
@@ -5378,7 +5378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>41</v>
       </c>
@@ -5404,7 +5404,7 @@
         <v>1.04</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -5427,7 +5427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -5450,7 +5450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>44</v>
       </c>
@@ -5476,7 +5476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>45</v>
       </c>
@@ -5499,7 +5499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>46</v>
       </c>
@@ -5525,7 +5525,7 @@
         <v>1.24</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>47</v>
       </c>
@@ -5548,7 +5548,7 @@
         <v>402.42815241375598</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>48</v>
       </c>
@@ -5574,7 +5574,7 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>49</v>
       </c>
@@ -5600,7 +5600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>50</v>
       </c>
@@ -5626,7 +5626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>51</v>
       </c>
@@ -5652,7 +5652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>52</v>
       </c>
@@ -5678,7 +5678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>53</v>
       </c>
@@ -5704,7 +5704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>54</v>
       </c>
@@ -5730,7 +5730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>55</v>
       </c>
@@ -5753,7 +5753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>56</v>
       </c>
@@ -5776,7 +5776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>57</v>
       </c>
@@ -5802,7 +5802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>58</v>
       </c>
@@ -5825,7 +5825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>59</v>
       </c>
@@ -5851,7 +5851,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>60</v>
       </c>
@@ -5877,7 +5877,7 @@
         <v>0.27</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>61</v>
       </c>
@@ -5903,7 +5903,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>62</v>
       </c>
@@ -5929,7 +5929,7 @@
         <v>0.21</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>63</v>
       </c>
@@ -5952,7 +5952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>64</v>
       </c>
@@ -5978,7 +5978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>65</v>
       </c>
@@ -6004,7 +6004,7 @@
         <v>0.62</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>66</v>
       </c>
@@ -6027,7 +6027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>67</v>
       </c>
@@ -6050,7 +6050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>68</v>
       </c>
@@ -6073,7 +6073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>69</v>
       </c>
@@ -6096,7 +6096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>70</v>
       </c>
@@ -6122,7 +6122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>71</v>
       </c>
@@ -6148,7 +6148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>72</v>
       </c>
@@ -6174,7 +6174,7 @@
         <v>0.77</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>73</v>
       </c>
@@ -6200,7 +6200,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>74</v>
       </c>
@@ -6223,7 +6223,7 @@
         <v>1.8399675063422279E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>75</v>
       </c>
@@ -6246,7 +6246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>76</v>
       </c>
@@ -6269,7 +6269,7 @@
         <v>2.1220275097995311</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>77</v>
       </c>
@@ -6292,7 +6292,7 @@
         <v>0.46577595243128161</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>78</v>
       </c>
@@ -6318,7 +6318,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>79</v>
       </c>
@@ -6344,7 +6344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>80</v>
       </c>
@@ -6370,7 +6370,7 @@
         <v>0.66</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>81</v>
       </c>
@@ -6404,13 +6404,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H75"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="6" max="6" width="15.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6436,7 +6436,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -6459,7 +6459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -6482,7 +6482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -6508,7 +6508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -6534,7 +6534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -6586,7 +6586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -6612,7 +6612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -6638,7 +6638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -6664,7 +6664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -6690,7 +6690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -6713,7 +6713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -6739,7 +6739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -6765,7 +6765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -6788,7 +6788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -6814,7 +6814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -6837,7 +6837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -6863,7 +6863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -6889,7 +6889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -6912,7 +6912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -6938,7 +6938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -6964,7 +6964,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -6990,7 +6990,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -7016,7 +7016,7 @@
         <v>0.27</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -7042,7 +7042,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>32</v>
       </c>
@@ -7065,7 +7065,7 @@
         <v>1960.1727230031829</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>33</v>
       </c>
@@ -7088,7 +7088,7 @@
         <v>1879.479684520212</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -7111,7 +7111,7 @@
         <v>2737.4563230780609</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>35</v>
       </c>
@@ -7134,7 +7134,7 @@
         <v>386.66514796748942</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>36</v>
       </c>
@@ -7160,7 +7160,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>37</v>
       </c>
@@ -7186,7 +7186,7 @@
         <v>0.19</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>38</v>
       </c>
@@ -7212,7 +7212,7 @@
         <v>0.21</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>39</v>
       </c>
@@ -7238,7 +7238,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>40</v>
       </c>
@@ -7264,7 +7264,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>41</v>
       </c>
@@ -7290,7 +7290,7 @@
         <v>0.68</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -7313,7 +7313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -7336,7 +7336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>44</v>
       </c>
@@ -7362,7 +7362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>45</v>
       </c>
@@ -7385,7 +7385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>46</v>
       </c>
@@ -7411,7 +7411,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>47</v>
       </c>
@@ -7434,7 +7434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>48</v>
       </c>
@@ -7460,7 +7460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>49</v>
       </c>
@@ -7486,7 +7486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>50</v>
       </c>
@@ -7512,7 +7512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>51</v>
       </c>
@@ -7538,7 +7538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>52</v>
       </c>
@@ -7564,7 +7564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>53</v>
       </c>
@@ -7590,7 +7590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>54</v>
       </c>
@@ -7616,7 +7616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>55</v>
       </c>
@@ -7639,7 +7639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>56</v>
       </c>
@@ -7662,7 +7662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>57</v>
       </c>
@@ -7688,7 +7688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>58</v>
       </c>
@@ -7711,7 +7711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>59</v>
       </c>
@@ -7737,7 +7737,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>60</v>
       </c>
@@ -7763,7 +7763,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>61</v>
       </c>
@@ -7789,7 +7789,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>62</v>
       </c>
@@ -7815,7 +7815,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>63</v>
       </c>
@@ -7838,7 +7838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>64</v>
       </c>
@@ -7864,7 +7864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>65</v>
       </c>
@@ -7890,7 +7890,7 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>66</v>
       </c>
@@ -7913,7 +7913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>67</v>
       </c>
@@ -7936,7 +7936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>68</v>
       </c>
@@ -7959,7 +7959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>69</v>
       </c>
@@ -7982,7 +7982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>70</v>
       </c>
@@ -8008,7 +8008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>71</v>
       </c>
@@ -8034,7 +8034,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>72</v>
       </c>
@@ -8060,7 +8060,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>73</v>
       </c>
@@ -8086,7 +8086,7 @@
         <v>0.72</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>74</v>
       </c>
@@ -8109,7 +8109,7 @@
         <v>9.1998375317111376E-3</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>75</v>
       </c>
@@ -8132,7 +8132,7 @@
         <v>0.1465212026018109</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>76</v>
       </c>
@@ -8155,7 +8155,7 @@
         <v>0.2789866537631337</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>77</v>
       </c>
@@ -8178,7 +8178,7 @@
         <v>2.1695066233766609E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>78</v>
       </c>
@@ -8204,7 +8204,7 @@
         <v>0.69</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>79</v>
       </c>
@@ -8230,7 +8230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>80</v>
       </c>
@@ -8256,7 +8256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>81</v>
       </c>
@@ -8290,9 +8290,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>82</v>
       </c>
@@ -8303,7 +8303,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -8314,7 +8314,7 @@
         <v>137813</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>86</v>
       </c>
@@ -8325,7 +8325,7 @@
         <v>95068</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>87</v>
       </c>
@@ -8336,7 +8336,7 @@
         <v>186489</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>88</v>
       </c>
@@ -8355,16 +8355,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>82</v>
       </c>
@@ -8384,7 +8384,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -8404,7 +8404,7 @@
         <v>4803.696062957024</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>86</v>
       </c>
@@ -8424,7 +8424,7 @@
         <v>5269.5290770444872</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>87</v>
       </c>
@@ -8444,7 +8444,7 @@
         <v>12853.130391994249</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>88</v>
       </c>
@@ -8472,18 +8472,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.109375" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>97</v>
       </c>
@@ -8512,7 +8512,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>93</v>
       </c>
@@ -8538,7 +8538,7 @@
         <v>0.72</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>94</v>
       </c>
@@ -8564,7 +8564,7 @@
         <v>0.43</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>95</v>
       </c>
@@ -8590,11 +8590,11 @@
         <v>0.69</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -8623,7 +8623,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>39</v>
       </c>
@@ -8649,7 +8649,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>36</v>
       </c>
@@ -8675,7 +8675,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>38</v>
       </c>
@@ -8701,11 +8701,11 @@
         <v>0.68</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>99</v>
       </c>
@@ -8741,7 +8741,7 @@
         <v>-0.03</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C12">
         <f t="shared" ref="C12:I14" si="1">C7-C2</f>
         <v>610</v>
@@ -8771,7 +8771,7 @@
         <v>-0.25999999999999995</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C13">
         <f t="shared" si="1"/>
         <v>468</v>
@@ -8801,7 +8801,7 @@
         <v>-1.0000000000000009E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C14">
         <f t="shared" si="1"/>
         <v>621</v>
@@ -8831,7 +8831,7 @@
         <v>-9.9999999999998979E-3</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>97</v>
       </c>
@@ -8839,7 +8839,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
         <v>5</v>
       </c>
@@ -8850,7 +8850,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>92</v>
       </c>
@@ -8868,7 +8868,7 @@
         <v>3833376.1368651316</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>93</v>
       </c>
@@ -8886,7 +8886,7 @@
         <v>3250841.3018146493</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>94</v>
       </c>
@@ -8904,7 +8904,7 @@
         <v>1236899.9738707989</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>95</v>
       </c>
@@ -8931,14 +8931,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>82</v>
       </c>
@@ -8949,7 +8949,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -8960,7 +8960,7 @@
         <v>3840933</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>86</v>
       </c>
@@ -8971,7 +8971,7 @@
         <v>274320</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>87</v>
       </c>
@@ -8982,7 +8982,7 @@
         <v>676245</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>88</v>
       </c>
@@ -8993,25 +8993,25 @@
         <v>2915101</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C6" s="3"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>

</xml_diff>